<commit_message>
dataset mismatch errors working through for split
</commit_message>
<xml_diff>
--- a/house_labels.xlsx
+++ b/house_labels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilycastelan/Desktop/UMD/Spring26/MSLM640/-Image_Based_Classification_of_Residential_Exterior_Conditions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79CA8485-63F5-0E42-AC8B-7DD16E25F100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264CF5B1-8178-F041-9DF8-85B0231EEA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9780" yWindow="6760" windowWidth="18860" windowHeight="11460" xr2:uid="{E02F489E-0FFA-7147-A741-D82A0AA64D27}"/>
+    <workbookView xWindow="3420" yWindow="740" windowWidth="25220" windowHeight="17480" xr2:uid="{E02F489E-0FFA-7147-A741-D82A0AA64D27}"/>
   </bookViews>
   <sheets>
     <sheet name="house_labels" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="89">
   <si>
     <t>image_number</t>
   </si>
@@ -294,126 +294,6 @@
   </si>
   <si>
     <t>img_079</t>
-  </si>
-  <si>
-    <t>img_080</t>
-  </si>
-  <si>
-    <t>img_081</t>
-  </si>
-  <si>
-    <t>img_082</t>
-  </si>
-  <si>
-    <t>img_083</t>
-  </si>
-  <si>
-    <t>img_084</t>
-  </si>
-  <si>
-    <t>img_085</t>
-  </si>
-  <si>
-    <t>img_086</t>
-  </si>
-  <si>
-    <t>img_087</t>
-  </si>
-  <si>
-    <t>img_088</t>
-  </si>
-  <si>
-    <t>img_089</t>
-  </si>
-  <si>
-    <t>img_090</t>
-  </si>
-  <si>
-    <t>img_091</t>
-  </si>
-  <si>
-    <t>img_092</t>
-  </si>
-  <si>
-    <t>img_093</t>
-  </si>
-  <si>
-    <t>img_094</t>
-  </si>
-  <si>
-    <t>img_095</t>
-  </si>
-  <si>
-    <t>img_096</t>
-  </si>
-  <si>
-    <t>img_097</t>
-  </si>
-  <si>
-    <t>img_098</t>
-  </si>
-  <si>
-    <t>img_099</t>
-  </si>
-  <si>
-    <t>img_100</t>
-  </si>
-  <si>
-    <t>img_101</t>
-  </si>
-  <si>
-    <t>img_102</t>
-  </si>
-  <si>
-    <t>img_103</t>
-  </si>
-  <si>
-    <t>img_104</t>
-  </si>
-  <si>
-    <t>img_105</t>
-  </si>
-  <si>
-    <t>img_106</t>
-  </si>
-  <si>
-    <t>img_107</t>
-  </si>
-  <si>
-    <t>img_108</t>
-  </si>
-  <si>
-    <t>img_109</t>
-  </si>
-  <si>
-    <t>img_110</t>
-  </si>
-  <si>
-    <t>img_111</t>
-  </si>
-  <si>
-    <t>img_112</t>
-  </si>
-  <si>
-    <t>img_113</t>
-  </si>
-  <si>
-    <t>img_114</t>
-  </si>
-  <si>
-    <t>img_115</t>
-  </si>
-  <si>
-    <t>img_116</t>
-  </si>
-  <si>
-    <t>img_117</t>
-  </si>
-  <si>
-    <t>img_118</t>
-  </si>
-  <si>
-    <t>img_119</t>
   </si>
   <si>
     <t>poor</t>
@@ -800,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56F469DE-47FB-FF43-9F4C-D93E3658C075}">
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -846,7 +726,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -869,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -892,7 +772,7 @@
         <v>6</v>
       </c>
       <c r="G4" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -915,7 +795,7 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -938,7 +818,7 @@
         <v>7</v>
       </c>
       <c r="G6" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -962,7 +842,7 @@
         <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -986,7 +866,7 @@
         <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1010,7 +890,7 @@
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1034,7 +914,7 @@
         <v>8</v>
       </c>
       <c r="G10" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1058,7 +938,7 @@
         <v>8</v>
       </c>
       <c r="G11" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1082,7 +962,7 @@
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1106,7 +986,7 @@
         <v>4</v>
       </c>
       <c r="G13" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1130,7 +1010,7 @@
         <v>3</v>
       </c>
       <c r="G14" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1154,7 +1034,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1178,7 +1058,7 @@
         <v>8</v>
       </c>
       <c r="G16" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1202,7 +1082,7 @@
         <v>6</v>
       </c>
       <c r="G17" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1226,7 +1106,7 @@
         <v>4</v>
       </c>
       <c r="G18" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1250,7 +1130,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1274,7 +1154,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1298,7 +1178,7 @@
         <v>4</v>
       </c>
       <c r="G21" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1322,7 +1202,7 @@
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1346,7 +1226,7 @@
         <v>4</v>
       </c>
       <c r="G23" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1370,7 +1250,7 @@
         <v>3</v>
       </c>
       <c r="G24" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1394,7 +1274,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1418,7 +1298,7 @@
         <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1442,7 +1322,7 @@
         <v>5</v>
       </c>
       <c r="G27" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1466,7 +1346,7 @@
         <v>4</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1490,7 +1370,7 @@
         <v>5</v>
       </c>
       <c r="G29" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1514,7 +1394,7 @@
         <v>6</v>
       </c>
       <c r="G30" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1538,7 +1418,7 @@
         <v>4</v>
       </c>
       <c r="G31" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1562,7 +1442,7 @@
         <v>6</v>
       </c>
       <c r="G32" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1586,7 +1466,7 @@
         <v>6</v>
       </c>
       <c r="G33" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1610,7 +1490,7 @@
         <v>8</v>
       </c>
       <c r="G34" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1634,7 +1514,7 @@
         <v>7</v>
       </c>
       <c r="G35" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1658,7 +1538,7 @@
         <v>8</v>
       </c>
       <c r="G36" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1682,7 +1562,7 @@
         <v>2</v>
       </c>
       <c r="G37" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1706,7 +1586,7 @@
         <v>3</v>
       </c>
       <c r="G38" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1730,7 +1610,7 @@
         <v>1</v>
       </c>
       <c r="G39" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1754,7 +1634,7 @@
         <v>1</v>
       </c>
       <c r="G40" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1778,7 +1658,7 @@
         <v>2</v>
       </c>
       <c r="G41" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1802,7 +1682,7 @@
         <v>2</v>
       </c>
       <c r="G42" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1826,7 +1706,7 @@
         <v>2</v>
       </c>
       <c r="G43" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1850,7 +1730,7 @@
         <v>4</v>
       </c>
       <c r="G44" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1874,7 +1754,7 @@
         <v>4</v>
       </c>
       <c r="G45" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1898,7 +1778,7 @@
         <v>6</v>
       </c>
       <c r="G46" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1922,7 +1802,7 @@
         <v>5</v>
       </c>
       <c r="G47" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1946,7 +1826,7 @@
         <v>4</v>
       </c>
       <c r="G48" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1970,7 +1850,7 @@
         <v>5</v>
       </c>
       <c r="G49" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1994,7 +1874,7 @@
         <v>6</v>
       </c>
       <c r="G50" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -2018,7 +1898,7 @@
         <v>4</v>
       </c>
       <c r="G51" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -2042,7 +1922,7 @@
         <v>6</v>
       </c>
       <c r="G52" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -2066,7 +1946,7 @@
         <v>8</v>
       </c>
       <c r="G53" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -2090,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="G54" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -2114,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="G55" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -2138,7 +2018,7 @@
         <v>8</v>
       </c>
       <c r="G56" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -2162,7 +2042,7 @@
         <v>8</v>
       </c>
       <c r="G57" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -2186,7 +2066,7 @@
         <v>8</v>
       </c>
       <c r="G58" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -2210,7 +2090,7 @@
         <v>7</v>
       </c>
       <c r="G59" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -2234,7 +2114,7 @@
         <v>8</v>
       </c>
       <c r="G60" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -2258,7 +2138,7 @@
         <v>8</v>
       </c>
       <c r="G61" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -2282,7 +2162,7 @@
         <v>8</v>
       </c>
       <c r="G62" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -2306,7 +2186,7 @@
         <v>8</v>
       </c>
       <c r="G63" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2330,7 +2210,7 @@
         <v>7</v>
       </c>
       <c r="G64" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
@@ -2354,7 +2234,7 @@
         <v>3</v>
       </c>
       <c r="G65" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2378,7 +2258,7 @@
         <v>3</v>
       </c>
       <c r="G66" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2402,7 +2282,7 @@
         <v>3</v>
       </c>
       <c r="G67" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2426,7 +2306,7 @@
         <v>3</v>
       </c>
       <c r="G68" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -2450,7 +2330,7 @@
         <v>1</v>
       </c>
       <c r="G69" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2474,7 +2354,7 @@
         <v>3</v>
       </c>
       <c r="G70" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2498,7 +2378,7 @@
         <v>5</v>
       </c>
       <c r="G71" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2522,7 +2402,7 @@
         <v>6</v>
       </c>
       <c r="G72" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2546,7 +2426,7 @@
         <v>5</v>
       </c>
       <c r="G73" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -2570,7 +2450,7 @@
         <v>3</v>
       </c>
       <c r="G74" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -2594,7 +2474,7 @@
         <v>4</v>
       </c>
       <c r="G75" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -2618,7 +2498,7 @@
         <v>5</v>
       </c>
       <c r="G76" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
@@ -2642,7 +2522,7 @@
         <v>7</v>
       </c>
       <c r="G77" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
@@ -2666,7 +2546,7 @@
         <v>8</v>
       </c>
       <c r="G78" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2690,7 +2570,7 @@
         <v>7</v>
       </c>
       <c r="G79" t="s">
-        <v>128</v>
+        <v>88</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -2714,207 +2594,7 @@
         <v>7</v>
       </c>
       <c r="G80" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>